<commit_message>
docs: bs_service에 service_description 컬럼 추가 (설계서 §7.3 누락 보완)
CON-01 §8.3에서 필수 입력받는 '서비스 설명'이 §7.3 원본 DDL에는
누락되어 있어 코드(BsService 엔티티)와 불일치. 이를 보완:
- schema.sql: service_description varchar(300) NOT NULL 추가
- 별첨C 테이블설계서(BS_SERVICE 시트): 동일 컬럼 반영

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SLMxyQgKYFz74Rk29M4m6g
</commit_message>
<xml_diff>
--- a/docs/별첨C_테이블설계서.xlsx
+++ b/docs/별첨C_테이블설계서.xlsx
@@ -4078,7 +4078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4301,12 +4301,12 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>domain_code</t>
+          <t>service_description</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>varchar(30)</t>
+          <t>varchar(300)</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr"/>
@@ -4320,31 +4320,31 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F9" s="13" t="inlineStr">
-        <is>
-          <t>CLOSING, JOURNAL, EXPENSE, STATEMENT, CSM (파일럿 5개, 확장 가능)</t>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>업무 도메인 분류 코드(표시용)</t>
+          <t>서비스 설명(업무 목적). CON-01 §8.3 필수 항목</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>CLOSING</t>
+          <t>결산 단계별 상태 조회</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>service_type</t>
+          <t>domain_code</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>varchar(10)</t>
+          <t>varchar(30)</t>
         </is>
       </c>
       <c r="C10" s="12" t="inlineStr"/>
@@ -4360,29 +4360,29 @@
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
-          <t>READ(조회), ACTION(실행)  ※CHECK</t>
+          <t>CLOSING, JOURNAL, EXPENSE, STATEMENT, CSM (파일럿 5개, 확장 가능)</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>서비스 성격. 등록 시 값 검증에만 사용</t>
+          <t>업무 도메인 분류 코드(표시용)</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>READ</t>
+          <t>CLOSING</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>source_system</t>
+          <t>service_type</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>varchar(30)</t>
+          <t>varchar(10)</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr"/>
@@ -4393,34 +4393,34 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>'IFRS17'</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>IFRS17 (Phase1 기본·고정, 확장 가능)</t>
+          <t>READ(조회), ACTION(실행)  ※CHECK</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>서비스 원천 시스템(표시용)</t>
+          <t>서비스 성격. 등록 시 값 검증에만 사용</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>IFRS17</t>
+          <t>READ</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>owner_department</t>
+          <t>source_system</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>varchar(50)</t>
+          <t>varchar(30)</t>
         </is>
       </c>
       <c r="C12" s="12" t="inlineStr"/>
@@ -4431,34 +4431,34 @@
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>'IFRS17'</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>IFRS17 (Phase1 기본·고정, 확장 가능)</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>서비스 업무 책임 부서(Owner)</t>
+          <t>서비스 원천 시스템(표시용)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>정보기술팀</t>
+          <t>IFRS17</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>active_yn</t>
+          <t>owner_department</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>char(1)</t>
+          <t>varchar(50)</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr"/>
@@ -4469,34 +4469,34 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>'Y'</t>
-        </is>
-      </c>
-      <c r="F13" s="13" t="inlineStr">
-        <is>
-          <t>Y(사용), N(미사용)</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>서비스 사용 여부(N이면 신규 호출 즉시 차단) [핵심 로직]</t>
+          <t>서비스 업무 책임 부서(Owner)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>정보기술팀</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>active_yn</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>timestamp</t>
+          <t>char(1)</t>
         </is>
       </c>
       <c r="C14" s="12" t="inlineStr"/>
@@ -4507,34 +4507,34 @@
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>current_timestamp</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>'Y'</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>Y(사용), N(미사용)</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>최초 등록 일시(감사)</t>
+          <t>서비스 사용 여부(N이면 신규 호출 즉시 차단) [핵심 로직]</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>2026-07-14 09:00:00</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>created_by</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>varchar(30)</t>
+          <t>timestamp</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr"/>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>current_timestamp</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -4555,24 +4555,24 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>최초 등록자 ID(감사)</t>
+          <t>최초 등록 일시(감사)</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>E12345</t>
+          <t>2026-07-14 09:00:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>created_by</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>timestamp</t>
+          <t>varchar(30)</t>
         </is>
       </c>
       <c r="C16" s="12" t="inlineStr"/>
@@ -4583,7 +4583,7 @@
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>current_timestamp</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -4593,24 +4593,24 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>최종 수정 일시(감사)</t>
+          <t>최초 등록자 ID(감사)</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:00</t>
+          <t>E12345</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>updated_by</t>
+          <t>updated_at</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>varchar(30)</t>
+          <t>timestamp</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr"/>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>current_timestamp</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -4631,17 +4631,55 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
+          <t>최종 수정 일시(감사)</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-30 10:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>updated_by</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>varchar(30)</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr"/>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
           <t>최종 수정자 ID(감사)</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>E12345</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="14" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
         <is>
           <t>범례: 유효값(코드값) 열=코드성 컬럼만 기재(연녹 음영) · PK 컬럼 음영 · [핵심 로직]=실행/조회 분기에 사용 · '-'=자유값/해당없음</t>
         </is>
@@ -4652,7 +4690,7 @@
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="G2:H2"/>
-    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A20:H20"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="A1:H1"/>

</xml_diff>

<commit_message>
docs: 권한 설계 상세화 - BS_SERVICE_ROLE.role_code를 '화면ID:액션' 형식으로 확정
역할코드 기반 → 화면/액션 기반 권한으로 상세화(외부 권한API 모델 반영):
- role_code 형식: 화면ID:액션 (콜론 구분)
  · 화면ID = [A-Z]{4}M[0-9]{3} (예: CLSGM001)
  · 액션 = inqy(조회)/sv(저장)/cnfr(확정)/aprl(승인)/prt(출력)
- 판정: 외부 권한API의 사용자 화면권한(Y/N)과 AND 비교
- 별첨C: BS_SERVICE_ROLE 유효값/용도 갱신 + 목록시트 사용여부 '사용' 확정
- schema.sql: role_code 형식 주석 보강 (구조 변경 없음)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SLMxyQgKYFz74Rk29M4m6g
</commit_message>
<xml_diff>
--- a/docs/별첨C_테이블설계서.xlsx
+++ b/docs/별첨C_테이블설계서.xlsx
@@ -764,17 +764,17 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>서비스 역할 권한</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>미확정</t>
+          <t>서비스 필요 권한</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>사용</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>서비스 호출에 필요한 허용 역할(§6.2 권한 원칙, §8.3 허용 역할)</t>
+          <t>서비스 호출에 필요한 권한(화면ID:액션). 외부 권한API의 사용자 화면권한과 AND 비교(§6.2 권한 원칙)</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>상세설계서 v1.3 §7.2 (신규)</t>
+          <t>상세설계서 v1.3 §7.2 (신규) + 권한설계 상세화</t>
         </is>
       </c>
     </row>
@@ -5818,7 +5818,7 @@
       </c>
       <c r="G2" s="12" t="inlineStr">
         <is>
-          <t>서비스 역할 권한</t>
+          <t>서비스 필요 권한</t>
         </is>
       </c>
       <c r="H2" s="12" t="n"/>
@@ -5857,7 +5857,7 @@
       </c>
       <c r="B4" s="12" t="inlineStr">
         <is>
-          <t>서비스 호출에 필요한 허용 역할(§6.2 권한 원칙, §8.3 허용 역할)</t>
+          <t>서비스 호출에 필요한 권한(화면ID:액션). 외부 권한API의 사용자 화면권한과 AND 비교(§6.2 권한 원칙)</t>
         </is>
       </c>
       <c r="C4" s="12" t="n"/>
@@ -5870,7 +5870,7 @@
       </c>
       <c r="G4" s="12" t="inlineStr">
         <is>
-          <t>상세설계서 v1.3 §7.2 (신규)</t>
+          <t>상세설계서 v1.3 §7.2 (신규) + 권한설계 상세화</t>
         </is>
       </c>
       <c r="H4" s="12" t="n"/>
@@ -5985,19 +5985,19 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="F8" s="16" t="inlineStr">
+        <is>
+          <t>화면ID:액션 형식  ·  화면ID=[A-Z]{4}M[0-9]{3}  ·  액션=inqy(조회)/sv(저장)/cnfr(확정)/aprl(승인)/prt(출력)</t>
         </is>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
-          <t>허용 역할 코드(IFRS17 권한체계 기준)</t>
+          <t>필요 권한 코드(화면ID:액션). 외부 권한API의 사용자 화면권한(Y/N)과 AND 비교</t>
         </is>
       </c>
       <c r="H8" s="14" t="inlineStr">
         <is>
-          <t>IFRS17_CLOSING_VIEW</t>
+          <t>CLSGM001:inqy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: BS_CLIENT.client_id 명명 규칙 정의 반영
client_id 값 규칙을 '{채널}-{시스템}-{일련번호}'로 정의(설계서 §5.2
예시 MCP-IFRS17-01 기반):
- 정규식 [A-Z0-9]+-[A-Z0-9]+-[0-9]{2}, 채널은 하이픈 없는 코드
- schema.sql 주석 + 별첨C BS_CLIENT client_id 유효값 반영

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SLMxyQgKYFz74Rk29M4m6g
</commit_message>
<xml_diff>
--- a/docs/별첨C_테이블설계서.xlsx
+++ b/docs/별첨C_테이블설계서.xlsx
@@ -6271,14 +6271,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>형식 {채널}-{시스템}-{일련번호}  ·  정규식 [A-Z0-9]+-[A-Z0-9]+-[0-9]{2}  ·  채널은 하이픈 없는 코드</t>
         </is>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
-          <t>호출 Client 식별자(X-Client-ID) [핵심 로직]</t>
+          <t>호출 Client 식별자(X-Client-ID). 명명규칙 {채널}-{시스템}-{일련번호} [핵심 로직]</t>
         </is>
       </c>
       <c r="H7" s="14" t="inlineStr">

</xml_diff>

<commit_message>
docs: BS_CLIENT_SERVICE 사용 여부 '사용'으로 확정
ClientValidator에서 Client×서비스 허용 인가에 실제 사용됨 확인.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SLMxyQgKYFz74Rk29M4m6g
</commit_message>
<xml_diff>
--- a/docs/별첨C_테이블설계서.xlsx
+++ b/docs/별첨C_테이블설계서.xlsx
@@ -837,9 +837,9 @@
           <t>Client별 호출 허용</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>미확정</t>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>사용</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs: BS_CALL_LOG 감사 무결성 보강 (request_id 서버생성 + client_request_id 추가)
호출자가 중복 X-Request-ID를 보내면 기존 감사로그가 덮어써지는 위험을
문서에 반영 (코드 미변경, 문서 확정만):
- request_id(PK)는 서버 생성 유일값으로 정의(호출자 헤더 미사용)
- client_request_id 컬럼 신규(호출자 X-Request-ID 원본, 추적·상관용)
- 생성형식: 시각+시퀀스/UUID 조합(기존 %10000 순환 대체)
- schema.sql 주석 + 별첨C BS_CALL_LOG(18→19컬럼) 반영

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SLMxyQgKYFz74Rk29M4m6g
</commit_message>
<xml_diff>
--- a/docs/별첨C_테이블설계서.xlsx
+++ b/docs/별첨C_테이블설계서.xlsx
@@ -879,7 +879,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>서비스 호출 감사로그(§6.3 감사 필수항목)</t>
+          <t>서비스 호출 감사로그(§6.3). request_id(PK)는 서버 생성 유일값, 호출자 X-Request-ID는 client_request_id에 별도 저장(무결성)</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>상세설계서 v1.3 §7.3 (원본)</t>
+          <t>상세설계서 v1.3 §7.3 (원본) + 감사 무결성 보강</t>
         </is>
       </c>
     </row>
@@ -6905,7 +6905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6985,7 +6985,7 @@
       </c>
       <c r="B4" s="12" t="inlineStr">
         <is>
-          <t>서비스 호출 감사로그(§6.3 감사 필수항목)</t>
+          <t>서비스 호출 감사로그(§6.3). request_id(PK)는 서버 생성 유일값, 호출자 X-Request-ID는 client_request_id에 별도 저장(무결성)</t>
         </is>
       </c>
       <c r="C4" s="12" t="n"/>
@@ -6998,7 +6998,7 @@
       </c>
       <c r="G4" s="12" t="inlineStr">
         <is>
-          <t>상세설계서 v1.3 §7.3 (원본)</t>
+          <t>상세설계서 v1.3 §7.3 (원본) + 감사 무결성 보강</t>
         </is>
       </c>
       <c r="H4" s="12" t="n"/>
@@ -7078,19 +7078,19 @@
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
-          <t>호출 요청 고유 ID</t>
+          <t>호출 요청 고유 ID — 서버 생성 유일값(호출자 헤더 미사용). 코드 반영 예정 [핵심 로직]</t>
         </is>
       </c>
       <c r="H7" s="14" t="inlineStr">
         <is>
-          <t>REQ-20260714-0001</t>
+          <t>REQ-20260714093012345-1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>trace_id</t>
+          <t>client_request_id</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -7112,32 +7112,28 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>분산추적 ID</t>
+          <t>[신규] 호출자 X-Request-ID 원본(추적·상관용, 유일성 미보장·중복 가능)</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>TRACE-abc123</t>
+          <t>REQ-20260714-0001</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>service_id</t>
+          <t>trace_id</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>varchar(100)</t>
+          <t>varchar(80)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D9" s="4" t="inlineStr"/>
       <c r="E9" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -7150,24 +7146,24 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>호출 서비스 ID</t>
+          <t>분산추적 ID</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>IFRS17.CLOSING.STATUS</t>
+          <t>TRACE-abc123</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>service_version</t>
+          <t>service_id</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>varchar(20)</t>
+          <t>varchar(100)</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr"/>
@@ -7188,24 +7184,24 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>호출 서비스 버전</t>
+          <t>호출 서비스 ID</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>IFRS17.CLOSING.STATUS</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>client_id</t>
+          <t>service_version</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>varchar(80)</t>
+          <t>varchar(20)</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr"/>
@@ -7226,28 +7222,32 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>호출 Client ID</t>
+          <t>호출 서비스 버전</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>MCP-IFRS17-01</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>user_id</t>
+          <t>client_id</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>varchar(50)</t>
+          <t>varchar(80)</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr"/>
-      <c r="D12" s="4" t="inlineStr"/>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -7260,19 +7260,19 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>사용자 ID(대리호출 시 실사용자)</t>
+          <t>호출 Client ID</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>E12345</t>
+          <t>MCP-IFRS17-01</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>department_code</t>
+          <t>user_id</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -7294,32 +7294,28 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>사용자 부서 코드</t>
+          <t>사용자 ID(대리호출 시 실사용자)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>FIN01</t>
+          <t>E12345</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>requested_at</t>
+          <t>department_code</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>timestamp</t>
+          <t>varchar(50)</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr"/>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D14" s="4" t="inlineStr"/>
       <c r="E14" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -7332,19 +7328,19 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>요청 수신 일시</t>
+          <t>사용자 부서 코드</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>2026-07-14 09:00:00</t>
+          <t>FIN01</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>completed_at</t>
+          <t>requested_at</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -7353,7 +7349,11 @@
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr"/>
-      <c r="D15" s="4" t="inlineStr"/>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -7366,24 +7366,24 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>처리 완료 일시</t>
+          <t>요청 수신 일시</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>2026-07-14 09:00:01</t>
+          <t>2026-07-14 09:00:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>elapsed_ms</t>
+          <t>completed_at</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>timestamp</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr"/>
@@ -7400,66 +7400,66 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>처리 소요시간(ms)</t>
+          <t>처리 완료 일시</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>850</t>
+          <t>2026-07-14 09:00:01</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>status_code</t>
+          <t>elapsed_ms</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>varchar(20)</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr"/>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D17" s="4" t="inlineStr"/>
       <c r="E17" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F17" s="16" t="inlineStr">
-        <is>
-          <t>COMPLETED, PARTIAL, FAILED 등 (부록D)</t>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>처리 상태</t>
+          <t>처리 소요시간(ms)</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>COMPLETED</t>
+          <t>850</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>http_status</t>
+          <t>status_code</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>varchar(20)</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="4" t="inlineStr"/>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -7467,29 +7467,29 @@
       </c>
       <c r="F18" s="16" t="inlineStr">
         <is>
-          <t>200, 400, 401, 403, 404, 500 등</t>
+          <t>COMPLETED, PARTIAL, FAILED 등 (부록D)</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>HTTP 상태코드</t>
+          <t>처리 상태</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>COMPLETED</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>error_code</t>
+          <t>http_status</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>varchar(50)</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr"/>
@@ -7501,29 +7501,29 @@
       </c>
       <c r="F19" s="16" t="inlineStr">
         <is>
-          <t>BS-VAL-001, BS-AUTH-003 등 (부록A)</t>
+          <t>200, 400, 401, 403, 404, 500 등</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>오류코드</t>
+          <t>HTTP 상태코드</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>BS-VAL-001</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>error_id</t>
+          <t>error_code</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>varchar(80)</t>
+          <t>varchar(50)</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr"/>
@@ -7533,31 +7533,31 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="F20" s="16" t="inlineStr">
+        <is>
+          <t>BS-VAL-001, BS-AUTH-003 등 (부록A)</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>오류 추적 ID</t>
+          <t>오류코드</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>ERR-xyz789</t>
+          <t>BS-VAL-001</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>parameter_hash</t>
+          <t>error_id</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>varchar(128)</t>
+          <t>varchar(80)</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr"/>
@@ -7574,24 +7574,24 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>요청 파라미터 Hash(원문 저장 금지)</t>
+          <t>오류 추적 ID</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>a1b2c3...</t>
+          <t>ERR-xyz789</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>result_count</t>
+          <t>parameter_hash</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>varchar(128)</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr"/>
@@ -7608,24 +7608,24 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>결과 건수</t>
+          <t>요청 파라미터 Hash(원문 저장 금지)</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>a1b2c3...</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>remote_ip</t>
+          <t>result_count</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>varchar(64)</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr"/>
@@ -7642,24 +7642,24 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>호출 원격 IP</t>
+          <t>결과 건수</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>10.1.2.3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>server_instance</t>
+          <t>remote_ip</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>varchar(100)</t>
+          <t>varchar(64)</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr"/>
@@ -7676,17 +7676,51 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
+          <t>호출 원격 IP</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>10.1.2.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>server_instance</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>varchar(100)</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr"/>
+      <c r="D25" s="4" t="inlineStr"/>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
           <t>처리 WAS 인스턴스</t>
         </is>
       </c>
-      <c r="H24" s="5" t="inlineStr">
+      <c r="H25" s="5" t="inlineStr">
         <is>
           <t>was-01</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>범례: 유효값(코드값) 열=코드성 컬럼만 기재(연녹 음영) · PK 컬럼 음영 · [핵심 로직]=실행/조회 분기에 사용 · '-'=자유값/해당없음</t>
         </is>
@@ -7695,12 +7729,12 @@
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="G4:H4"/>
-    <mergeCell ref="A26:H26"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A27:H27"/>
     <mergeCell ref="G3:H3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs: BS_SERVICE_DEPLOYMENT 사용 여부 '미사용(미구현)'으로 확정
§8.1에서 배포관리·JAR 업로드는 Phase 1 범위 제외로 명시. 엔티티/코드
미구현. Bean 검증은 ServiceSpecService.validateBean이 실시간 처리.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SLMxyQgKYFz74Rk29M4m6g
</commit_message>
<xml_diff>
--- a/docs/별첨C_테이블설계서.xlsx
+++ b/docs/별첨C_테이블설계서.xlsx
@@ -1035,9 +1035,9 @@
           <t>배포 구현체 정보</t>
         </is>
       </c>
-      <c r="D15" s="11" t="inlineStr">
-        <is>
-          <t>미확정</t>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>미사용(미구현)</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs: BS_SERVICE_APPROVAL 사용 여부 '미사용(미구현)'으로 확정
§8.1에서 복잡한 승인 Workflow는 Phase 1 범위 제외로 명시. 엔티티/코드
미구현. 현재 콘솔은 저장 즉시 반영(승인 단계 없음).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SLMxyQgKYFz74Rk29M4m6g
</commit_message>
<xml_diff>
--- a/docs/별첨C_테이블설계서.xlsx
+++ b/docs/별첨C_테이블설계서.xlsx
@@ -1070,9 +1070,9 @@
           <t>등록·변경·활성화 승인 이력</t>
         </is>
       </c>
-      <c r="D16" s="11" t="inlineStr">
-        <is>
-          <t>미확정</t>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>미사용(미구현)</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs: BS_SERVICE_CHANGE_LOG 사용 여부 '미사용(미구현)'으로 확정
필드 단위 전/후 변경로그. 엔티티/코드 미구현. 상위 개념
BS_CHANGE_HISTORY도 미사용이므로 함께 미사용 확정.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SLMxyQgKYFz74Rk29M4m6g
</commit_message>
<xml_diff>
--- a/docs/별첨C_테이블설계서.xlsx
+++ b/docs/별첨C_테이블설계서.xlsx
@@ -1105,9 +1105,9 @@
           <t>메타데이터 변경 전/후 이력</t>
         </is>
       </c>
-      <c r="D17" s="11" t="inlineStr">
-        <is>
-          <t>미확정</t>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>미사용(미구현)</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs: BS_SERVICE_CACHE_EVENT 사용 여부 '미사용(미구현)'으로 확정
다중 WAS 캐시 무효화 이벤트. 현재 메타데이터는 매번 DB 조회로 캐시
계층 자체가 없어 무효화 대상 없음. 엔티티/코드 미구현. 14개 테이블
사용 여부 검토 완료.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SLMxyQgKYFz74Rk29M4m6g
</commit_message>
<xml_diff>
--- a/docs/별첨C_테이블설계서.xlsx
+++ b/docs/별첨C_테이블설계서.xlsx
@@ -31,7 +31,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -87,18 +87,12 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="009C0006"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
     </font>
     <font>
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -133,11 +127,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -187,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -219,28 +208,25 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1140,9 +1126,9 @@
           <t>다중 WAS Cache 무효화 이벤트</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
-        <is>
-          <t>미확정</t>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>미사용(미구현)</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1162,7 +1148,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="inlineStr">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>사용 여부 범례: 사용=코드에서 실제 사용 · 미사용(정의만)=엔티티는 있으나 로직 미연결 · 미사용(미구현)=엔티티 없음 · 미사용(범위제외)=코드에 기록 로직 있으나 운영 범위 제외 · 미확정=공동 검토 전(코드 추정)</t>
         </is>
@@ -1205,162 +1191,162 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>테이블 ID</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>business_service.bs_change_history</t>
         </is>
       </c>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="13" t="inlineStr">
+      <c r="C2" s="13" t="n"/>
+      <c r="D2" s="13" t="n"/>
+      <c r="E2" s="13" t="n"/>
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>논리명</t>
         </is>
       </c>
-      <c r="G2" s="14" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>메타데이터 변경이력</t>
         </is>
       </c>
-      <c r="H2" s="14" t="n"/>
+      <c r="H2" s="13" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>주요 Key</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>change_id</t>
         </is>
       </c>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="12" t="inlineStr">
         <is>
           <t>DBMS</t>
         </is>
       </c>
-      <c r="G3" s="14" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>PostgreSQL</t>
         </is>
       </c>
-      <c r="H3" s="14" t="n"/>
+      <c r="H3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>메타데이터 변경 요약 이력(§7.4). ※코드에 recordChange 기록 로직 존재하나 운영 범위 제외(미사용)</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="14" t="n"/>
-      <c r="E4" s="14" t="n"/>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="13" t="n"/>
+      <c r="E4" s="13" t="n"/>
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>출처</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>상세설계서 v1.3 §7.2 (신규)</t>
         </is>
       </c>
-      <c r="H4" s="14" t="n"/>
+      <c r="H4" s="13" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>컬럼 ID</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>타입</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Not Null</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="F6" s="15" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>유효값(코드값)</t>
         </is>
       </c>
-      <c r="G6" s="15" t="inlineStr">
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>용도</t>
         </is>
       </c>
-      <c r="H6" s="15" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>예시</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>change_id</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>varchar(80)</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E7" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="16" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>변경 이력 ID</t>
         </is>
       </c>
-      <c r="H7" s="16" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
         <is>
           <t>CHG-0001</t>
         </is>
@@ -1388,7 +1374,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F8" s="18" t="inlineStr">
+      <c r="F8" s="17" t="inlineStr">
         <is>
           <t>SERVICE, VERSION, PARAM, ROLE, CLIENT 등</t>
         </is>
@@ -1464,7 +1450,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr">
+      <c r="F10" s="17" t="inlineStr">
         <is>
           <t>CREATE, UPDATE, DELETE, ACTIVATE, DEACTIVATE  ※CHECK</t>
         </is>
@@ -1591,7 +1577,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>범례: 유효값(코드값) 열=코드성 컬럼만 기재(연녹 음영) · PK 컬럼 음영 · [핵심 로직]=실행/조회 분기에 사용 · '-'=자유값/해당없음</t>
         </is>
@@ -1639,246 +1625,246 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>테이블 ID</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>business_service.bs_service_channel</t>
         </is>
       </c>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="13" t="inlineStr">
+      <c r="C2" s="13" t="n"/>
+      <c r="D2" s="13" t="n"/>
+      <c r="E2" s="13" t="n"/>
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>논리명</t>
         </is>
       </c>
-      <c r="G2" s="14" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>서비스별 허용 채널/Client 정책</t>
         </is>
       </c>
-      <c r="H2" s="14" t="n"/>
+      <c r="H2" s="13" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>주요 Key</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>service_id + version + channel_code</t>
         </is>
       </c>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="12" t="inlineStr">
         <is>
           <t>DBMS</t>
         </is>
       </c>
-      <c r="G3" s="14" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>PostgreSQL</t>
         </is>
       </c>
-      <c r="H3" s="14" t="n"/>
+      <c r="H3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>서비스 버전별 허용 채널과 Client 정책(§5.2, §6.2)</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="14" t="n"/>
-      <c r="E4" s="14" t="n"/>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="13" t="n"/>
+      <c r="E4" s="13" t="n"/>
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>출처</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>상세설계서 v1.3 §7.2 (신규)</t>
         </is>
       </c>
-      <c r="H4" s="14" t="n"/>
+      <c r="H4" s="13" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>컬럼 ID</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>타입</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Not Null</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="F6" s="15" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>유효값(코드값)</t>
         </is>
       </c>
-      <c r="G6" s="15" t="inlineStr">
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>용도</t>
         </is>
       </c>
-      <c r="H6" s="15" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>예시</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>service_id</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>varchar(100)</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E7" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="16" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>서비스 ID(FK→BS_SERVICE_VERSION)</t>
         </is>
       </c>
-      <c r="H7" s="16" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
         <is>
           <t>IFRS17.CLOSING.STATUS</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>varchar(20)</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D8" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E8" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G8" s="16" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
         <is>
           <t>서비스 버전(FK)</t>
         </is>
       </c>
-      <c r="H8" s="16" t="inlineStr">
+      <c r="H8" s="15" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>channel_code</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>varchar(30)</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D9" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E9" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F9" s="18" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="17" t="inlineStr">
         <is>
           <t>MCP, AI-AGENT, INTERNAL 등</t>
         </is>
       </c>
-      <c r="G9" s="16" t="inlineStr">
+      <c r="G9" s="15" t="inlineStr">
         <is>
           <t>허용 채널 코드</t>
         </is>
       </c>
-      <c r="H9" s="16" t="inlineStr">
+      <c r="H9" s="15" t="inlineStr">
         <is>
           <t>MCP</t>
         </is>
@@ -1906,7 +1892,7 @@
           <t>'Y'</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr">
+      <c r="F10" s="17" t="inlineStr">
         <is>
           <t>Y(허용), N(차단)</t>
         </is>
@@ -1944,7 +1930,7 @@
           <t>'ALLOWLIST'</t>
         </is>
       </c>
-      <c r="F11" s="18" t="inlineStr">
+      <c r="F11" s="17" t="inlineStr">
         <is>
           <t>ALLOWLIST, DENYLIST, OPEN  ※CHECK</t>
         </is>
@@ -2037,7 +2023,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>범례: 유효값(코드값) 열=코드성 컬럼만 기재(연녹 음영) · PK 컬럼 음영 · [핵심 로직]=실행/조회 분기에 사용 · '-'=자유값/해당없음</t>
         </is>
@@ -2085,162 +2071,162 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>테이블 ID</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>business_service.bs_service_deployment</t>
         </is>
       </c>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="13" t="inlineStr">
+      <c r="C2" s="13" t="n"/>
+      <c r="D2" s="13" t="n"/>
+      <c r="E2" s="13" t="n"/>
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>논리명</t>
         </is>
       </c>
-      <c r="G2" s="14" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>배포 구현체 정보</t>
         </is>
       </c>
-      <c r="H2" s="14" t="n"/>
+      <c r="H2" s="13" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>주요 Key</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>deployment_id</t>
         </is>
       </c>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="12" t="inlineStr">
         <is>
           <t>DBMS</t>
         </is>
       </c>
-      <c r="G3" s="14" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>PostgreSQL</t>
         </is>
       </c>
-      <c r="H3" s="14" t="n"/>
+      <c r="H3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>배포된 구현체·JAR/WAR·Bean·Checksum 정보(§8.4 배포·검증)</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="14" t="n"/>
-      <c r="E4" s="14" t="n"/>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="13" t="n"/>
+      <c r="E4" s="13" t="n"/>
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>출처</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>상세설계서 v1.3 §7.2 (신규)</t>
         </is>
       </c>
-      <c r="H4" s="14" t="n"/>
+      <c r="H4" s="13" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>컬럼 ID</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>타입</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Not Null</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="F6" s="15" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>유효값(코드값)</t>
         </is>
       </c>
-      <c r="G6" s="15" t="inlineStr">
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>용도</t>
         </is>
       </c>
-      <c r="H6" s="15" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>예시</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>deployment_id</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>varchar(80)</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E7" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="16" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>배포 이력 ID</t>
         </is>
       </c>
-      <c r="H7" s="16" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
         <is>
           <t>DEP-0001</t>
         </is>
@@ -2382,7 +2368,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F11" s="18" t="inlineStr">
+      <c r="F11" s="17" t="inlineStr">
         <is>
           <t>JAR, WAR  ※CHECK</t>
         </is>
@@ -2496,7 +2482,7 @@
           <t>'DEPLOYED'</t>
         </is>
       </c>
-      <c r="F14" s="18" t="inlineStr">
+      <c r="F14" s="17" t="inlineStr">
         <is>
           <t>DEPLOYED, VERIFIED, FAILED, RETIRED  ※CHECK</t>
         </is>
@@ -2534,7 +2520,7 @@
           <t>'N'</t>
         </is>
       </c>
-      <c r="F15" s="18" t="inlineStr">
+      <c r="F15" s="17" t="inlineStr">
         <is>
           <t>Y(검증완료), N(미검증)</t>
         </is>
@@ -2661,7 +2647,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="inlineStr">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>범례: 유효값(코드값) 열=코드성 컬럼만 기재(연녹 음영) · PK 컬럼 음영 · [핵심 로직]=실행/조회 분기에 사용 · '-'=자유값/해당없음</t>
         </is>
@@ -2709,162 +2695,162 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>테이블 ID</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>business_service.bs_service_approval</t>
         </is>
       </c>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="13" t="inlineStr">
+      <c r="C2" s="13" t="n"/>
+      <c r="D2" s="13" t="n"/>
+      <c r="E2" s="13" t="n"/>
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>논리명</t>
         </is>
       </c>
-      <c r="G2" s="14" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>등록·변경·활성화 승인 이력</t>
         </is>
       </c>
-      <c r="H2" s="14" t="n"/>
+      <c r="H2" s="13" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>주요 Key</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>approval_id</t>
         </is>
       </c>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="12" t="inlineStr">
         <is>
           <t>DBMS</t>
         </is>
       </c>
-      <c r="G3" s="14" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>PostgreSQL</t>
         </is>
       </c>
-      <c r="H3" s="14" t="n"/>
+      <c r="H3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>서비스 등록·변경·활성화 승인 이력(§6.2 운영자 승인, §8.4)</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="14" t="n"/>
-      <c r="E4" s="14" t="n"/>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="13" t="n"/>
+      <c r="E4" s="13" t="n"/>
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>출처</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>상세설계서 v1.3 §7.2 (신규)</t>
         </is>
       </c>
-      <c r="H4" s="14" t="n"/>
+      <c r="H4" s="13" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>컬럼 ID</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>타입</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Not Null</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="F6" s="15" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>유효값(코드값)</t>
         </is>
       </c>
-      <c r="G6" s="15" t="inlineStr">
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>용도</t>
         </is>
       </c>
-      <c r="H6" s="15" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>예시</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>approval_id</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>varchar(80)</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E7" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="16" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>승인 이력 ID</t>
         </is>
       </c>
-      <c r="H7" s="16" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
         <is>
           <t>APR-0001</t>
         </is>
@@ -2964,7 +2950,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr">
+      <c r="F10" s="17" t="inlineStr">
         <is>
           <t>REGISTER, MODIFY, ACTIVATE, DEACTIVATE  ※CHECK</t>
         </is>
@@ -3002,7 +2988,7 @@
           <t>'REQUESTED'</t>
         </is>
       </c>
-      <c r="F11" s="18" t="inlineStr">
+      <c r="F11" s="17" t="inlineStr">
         <is>
           <t>REQUESTED, APPROVED, REJECTED  ※CHECK</t>
         </is>
@@ -3197,7 +3183,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>범례: 유효값(코드값) 열=코드성 컬럼만 기재(연녹 음영) · PK 컬럼 음영 · [핵심 로직]=실행/조회 분기에 사용 · '-'=자유값/해당없음</t>
         </is>
@@ -3245,162 +3231,162 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>테이블 ID</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>business_service.bs_service_change_log</t>
         </is>
       </c>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="13" t="inlineStr">
+      <c r="C2" s="13" t="n"/>
+      <c r="D2" s="13" t="n"/>
+      <c r="E2" s="13" t="n"/>
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>논리명</t>
         </is>
       </c>
-      <c r="G2" s="14" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>메타데이터 변경 전/후 이력</t>
         </is>
       </c>
-      <c r="H2" s="14" t="n"/>
+      <c r="H2" s="13" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>주요 Key</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>change_id</t>
         </is>
       </c>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="12" t="inlineStr">
         <is>
           <t>DBMS</t>
         </is>
       </c>
-      <c r="G3" s="14" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>PostgreSQL</t>
         </is>
       </c>
-      <c r="H3" s="14" t="n"/>
+      <c r="H3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>메타데이터 필드 단위 변경 전/후 값 이력(BS_CHANGE_HISTORY는 요약)</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="14" t="n"/>
-      <c r="E4" s="14" t="n"/>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="13" t="n"/>
+      <c r="E4" s="13" t="n"/>
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>출처</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>상세설계서 v1.3 §7.2 (신규)</t>
         </is>
       </c>
-      <c r="H4" s="14" t="n"/>
+      <c r="H4" s="13" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>컬럼 ID</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>타입</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Not Null</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="F6" s="15" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>유효값(코드값)</t>
         </is>
       </c>
-      <c r="G6" s="15" t="inlineStr">
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>용도</t>
         </is>
       </c>
-      <c r="H6" s="15" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>예시</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>change_id</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>varchar(80)</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E7" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="16" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>변경 이력 ID</t>
         </is>
       </c>
-      <c r="H7" s="16" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
         <is>
           <t>CLG-0001</t>
         </is>
@@ -3699,7 +3685,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>범례: 유효값(코드값) 열=코드성 컬럼만 기재(연녹 음영) · PK 컬럼 음영 · [핵심 로직]=실행/조회 분기에 사용 · '-'=자유값/해당없음</t>
         </is>
@@ -3747,162 +3733,162 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>테이블 ID</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>business_service.bs_service_cache_event</t>
         </is>
       </c>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="13" t="inlineStr">
+      <c r="C2" s="13" t="n"/>
+      <c r="D2" s="13" t="n"/>
+      <c r="E2" s="13" t="n"/>
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>논리명</t>
         </is>
       </c>
-      <c r="G2" s="14" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>다중 WAS Cache 무효화 이벤트</t>
         </is>
       </c>
-      <c r="H2" s="14" t="n"/>
+      <c r="H2" s="13" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>주요 Key</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>event_id</t>
         </is>
       </c>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="12" t="inlineStr">
         <is>
           <t>DBMS</t>
         </is>
       </c>
-      <c r="G3" s="14" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>PostgreSQL</t>
         </is>
       </c>
-      <c r="H3" s="14" t="n"/>
+      <c r="H3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>다중 WAS 메타데이터 Cache 무효화 이벤트(§8.4 Registry 갱신)</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="14" t="n"/>
-      <c r="E4" s="14" t="n"/>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="13" t="n"/>
+      <c r="E4" s="13" t="n"/>
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>출처</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>상세설계서 v1.3 §7.2 (신규)</t>
         </is>
       </c>
-      <c r="H4" s="14" t="n"/>
+      <c r="H4" s="13" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>컬럼 ID</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>타입</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Not Null</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="F6" s="15" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>유효값(코드값)</t>
         </is>
       </c>
-      <c r="G6" s="15" t="inlineStr">
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>용도</t>
         </is>
       </c>
-      <c r="H6" s="15" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>예시</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>event_id</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>varchar(80)</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E7" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="16" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>캐시 이벤트 ID</t>
         </is>
       </c>
-      <c r="H7" s="16" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
         <is>
           <t>EVT-0001</t>
         </is>
@@ -3998,7 +3984,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr">
+      <c r="F10" s="17" t="inlineStr">
         <is>
           <t>INVALIDATE, RELOAD, EVICT_ALL  ※CHECK</t>
         </is>
@@ -4112,7 +4098,7 @@
           <t>'N'</t>
         </is>
       </c>
-      <c r="F13" s="18" t="inlineStr">
+      <c r="F13" s="17" t="inlineStr">
         <is>
           <t>Y(처리완료), N(미처리)</t>
         </is>
@@ -4197,7 +4183,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>범례: 유효값(코드값) 열=코드성 컬럼만 기재(연녹 음영) · PK 컬럼 음영 · [핵심 로직]=실행/조회 분기에 사용 · '-'=자유값/해당없음</t>
         </is>
@@ -4245,162 +4231,162 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>테이블 ID</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>business_service.bs_service</t>
         </is>
       </c>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="13" t="inlineStr">
+      <c r="C2" s="13" t="n"/>
+      <c r="D2" s="13" t="n"/>
+      <c r="E2" s="13" t="n"/>
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>논리명</t>
         </is>
       </c>
-      <c r="G2" s="14" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>서비스 Catalog</t>
         </is>
       </c>
-      <c r="H2" s="14" t="n"/>
+      <c r="H2" s="13" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>주요 Key</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>service_id</t>
         </is>
       </c>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="12" t="inlineStr">
         <is>
           <t>DBMS</t>
         </is>
       </c>
-      <c r="G3" s="14" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>PostgreSQL</t>
         </is>
       </c>
-      <c r="H3" s="14" t="n"/>
+      <c r="H3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Business Service 마스터(서비스 존재 등록). 버전·상태 세부는 BS_SERVICE_VERSION이 담당</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="14" t="n"/>
-      <c r="E4" s="14" t="n"/>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="13" t="n"/>
+      <c r="E4" s="13" t="n"/>
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>출처</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>상세설계서 v1.3 §7.3 (원본)</t>
         </is>
       </c>
-      <c r="H4" s="14" t="n"/>
+      <c r="H4" s="13" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>컬럼 ID</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>타입</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Not Null</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="F6" s="15" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>유효값(코드값)</t>
         </is>
       </c>
-      <c r="G6" s="15" t="inlineStr">
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>용도</t>
         </is>
       </c>
-      <c r="H6" s="15" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>예시</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>service_id</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>varchar(100)</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E7" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="16" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>서비스 고유 식별자(대문자·점 구분, 전역 유일, Handler ID와 일치). 실행/조회 조회키 [핵심 로직]</t>
         </is>
       </c>
-      <c r="H7" s="16" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
         <is>
           <t>IFRS17.CLOSING.STATUS</t>
         </is>
@@ -4504,7 +4490,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr">
+      <c r="F10" s="17" t="inlineStr">
         <is>
           <t>CLOSING, JOURNAL, EXPENSE, STATEMENT, CSM (파일럿 5개, 확장 가능)</t>
         </is>
@@ -4542,7 +4528,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F11" s="18" t="inlineStr">
+      <c r="F11" s="17" t="inlineStr">
         <is>
           <t>READ(조회), ACTION(실행)  ※CHECK</t>
         </is>
@@ -4580,7 +4566,7 @@
           <t>'IFRS17'</t>
         </is>
       </c>
-      <c r="F12" s="18" t="inlineStr">
+      <c r="F12" s="17" t="inlineStr">
         <is>
           <t>IFRS17 (Phase1 기본·고정, 확장 가능)</t>
         </is>
@@ -4656,7 +4642,7 @@
           <t>'Y'</t>
         </is>
       </c>
-      <c r="F14" s="18" t="inlineStr">
+      <c r="F14" s="17" t="inlineStr">
         <is>
           <t>Y(사용), N(미사용)</t>
         </is>
@@ -4825,7 +4811,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="inlineStr">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>범례: 유효값(코드값) 열=코드성 컬럼만 기재(연녹 음영) · PK 컬럼 음영 · [핵심 로직]=실행/조회 분기에 사용 · '-'=자유값/해당없음</t>
         </is>
@@ -4873,204 +4859,204 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>테이블 ID</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>business_service.bs_service_version</t>
         </is>
       </c>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="13" t="inlineStr">
+      <c r="C2" s="13" t="n"/>
+      <c r="D2" s="13" t="n"/>
+      <c r="E2" s="13" t="n"/>
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>논리명</t>
         </is>
       </c>
-      <c r="G2" s="14" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>서비스 버전</t>
         </is>
       </c>
-      <c r="H2" s="14" t="n"/>
+      <c r="H2" s="13" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>주요 Key</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>service_id + version</t>
         </is>
       </c>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="12" t="inlineStr">
         <is>
           <t>DBMS</t>
         </is>
       </c>
-      <c r="G3" s="14" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>PostgreSQL</t>
         </is>
       </c>
-      <c r="H3" s="14" t="n"/>
+      <c r="H3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>서비스의 버전별 상태·Schema·Timeout·구현 Bean 정의</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="14" t="n"/>
-      <c r="E4" s="14" t="n"/>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="13" t="n"/>
+      <c r="E4" s="13" t="n"/>
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>출처</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>상세설계서 v1.3 §7.3 (원본)</t>
         </is>
       </c>
-      <c r="H4" s="14" t="n"/>
+      <c r="H4" s="13" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>컬럼 ID</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>타입</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Not Null</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="F6" s="15" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>유효값(코드값)</t>
         </is>
       </c>
-      <c r="G6" s="15" t="inlineStr">
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>용도</t>
         </is>
       </c>
-      <c r="H6" s="15" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>예시</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>service_id</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>varchar(100)</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E7" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="16" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>서비스 ID(FK→BS_SERVICE)</t>
         </is>
       </c>
-      <c r="H7" s="16" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
         <is>
           <t>IFRS17.CLOSING.STATUS</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>varchar(20)</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D8" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E8" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G8" s="16" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
         <is>
           <t>서비스 버전</t>
         </is>
       </c>
-      <c r="H8" s="16" t="inlineStr">
+      <c r="H8" s="15" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
@@ -5242,7 +5228,7 @@
           <t>'ACTIVE'</t>
         </is>
       </c>
-      <c r="F13" s="18" t="inlineStr">
+      <c r="F13" s="17" t="inlineStr">
         <is>
           <t>ACTIVE(활성), INACTIVE(비활성)</t>
         </is>
@@ -5331,7 +5317,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>범례: 유효값(코드값) 열=코드성 컬럼만 기재(연녹 음영) · PK 컬럼 음영 · [핵심 로직]=실행/조회 분기에 사용 · '-'=자유값/해당없음</t>
         </is>
@@ -5379,246 +5365,246 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>테이블 ID</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>business_service.bs_service_param</t>
         </is>
       </c>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="13" t="inlineStr">
+      <c r="C2" s="13" t="n"/>
+      <c r="D2" s="13" t="n"/>
+      <c r="E2" s="13" t="n"/>
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>논리명</t>
         </is>
       </c>
-      <c r="G2" s="14" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>입력 파라미터 정의</t>
         </is>
       </c>
-      <c r="H2" s="14" t="n"/>
+      <c r="H2" s="13" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>주요 Key</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>service_id + version + param_name</t>
         </is>
       </c>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="12" t="inlineStr">
         <is>
           <t>DBMS</t>
         </is>
       </c>
-      <c r="G3" s="14" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>PostgreSQL</t>
         </is>
       </c>
-      <c r="H3" s="14" t="n"/>
+      <c r="H3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>서비스 버전별 입력 파라미터 명세(§8.3 요청 JSON 명세)</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="14" t="n"/>
-      <c r="E4" s="14" t="n"/>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="13" t="n"/>
+      <c r="E4" s="13" t="n"/>
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>출처</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>상세설계서 v1.3 §7.2 (신규)</t>
         </is>
       </c>
-      <c r="H4" s="14" t="n"/>
+      <c r="H4" s="13" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>컬럼 ID</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>타입</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Not Null</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="F6" s="15" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>유효값(코드값)</t>
         </is>
       </c>
-      <c r="G6" s="15" t="inlineStr">
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>용도</t>
         </is>
       </c>
-      <c r="H6" s="15" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>예시</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>service_id</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>varchar(100)</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E7" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="16" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>서비스 ID(FK→BS_SERVICE_VERSION)</t>
         </is>
       </c>
-      <c r="H7" s="16" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
         <is>
           <t>IFRS17.CLOSING.STATUS</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>varchar(20)</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D8" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E8" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G8" s="16" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
         <is>
           <t>서비스 버전(FK)</t>
         </is>
       </c>
-      <c r="H8" s="16" t="inlineStr">
+      <c r="H8" s="15" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>param_name</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>varchar(100)</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D9" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E9" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F9" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G9" s="16" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G9" s="15" t="inlineStr">
         <is>
           <t>파라미터 명</t>
         </is>
       </c>
-      <c r="H9" s="16" t="inlineStr">
+      <c r="H9" s="15" t="inlineStr">
         <is>
           <t>closingYearMonth</t>
         </is>
@@ -5646,7 +5632,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr">
+      <c r="F10" s="17" t="inlineStr">
         <is>
           <t>STRING, NUMBER, BOOLEAN, DATE 등</t>
         </is>
@@ -5684,7 +5670,7 @@
           <t>'Y'</t>
         </is>
       </c>
-      <c r="F11" s="18" t="inlineStr">
+      <c r="F11" s="17" t="inlineStr">
         <is>
           <t>Y(필수), N(선택)</t>
         </is>
@@ -5773,7 +5759,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>범례: 유효값(코드값) 열=코드성 컬럼만 기재(연녹 음영) · PK 컬럼 음영 · [핵심 로직]=실행/조회 분기에 사용 · '-'=자유값/해당없음</t>
         </is>
@@ -5821,204 +5807,204 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>테이블 ID</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>business_service.bs_service_role</t>
         </is>
       </c>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="13" t="inlineStr">
+      <c r="C2" s="13" t="n"/>
+      <c r="D2" s="13" t="n"/>
+      <c r="E2" s="13" t="n"/>
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>논리명</t>
         </is>
       </c>
-      <c r="G2" s="14" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>서비스 필요 권한</t>
         </is>
       </c>
-      <c r="H2" s="14" t="n"/>
+      <c r="H2" s="13" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>주요 Key</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>service_id + role_code</t>
         </is>
       </c>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="12" t="inlineStr">
         <is>
           <t>DBMS</t>
         </is>
       </c>
-      <c r="G3" s="14" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>PostgreSQL</t>
         </is>
       </c>
-      <c r="H3" s="14" t="n"/>
+      <c r="H3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>서비스 호출에 필요한 권한(화면ID:액션). 외부 권한API의 사용자 화면권한과 AND 비교(§6.2 권한 원칙)</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="14" t="n"/>
-      <c r="E4" s="14" t="n"/>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="13" t="n"/>
+      <c r="E4" s="13" t="n"/>
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>출처</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>상세설계서 v1.3 §7.2 (신규) + 권한설계 상세화</t>
         </is>
       </c>
-      <c r="H4" s="14" t="n"/>
+      <c r="H4" s="13" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>컬럼 ID</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>타입</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Not Null</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="F6" s="15" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>유효값(코드값)</t>
         </is>
       </c>
-      <c r="G6" s="15" t="inlineStr">
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>용도</t>
         </is>
       </c>
-      <c r="H6" s="15" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>예시</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>service_id</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>varchar(100)</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E7" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="16" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>서비스 ID(FK→BS_SERVICE)</t>
         </is>
       </c>
-      <c r="H7" s="16" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
         <is>
           <t>IFRS17.CLOSING.STATUS</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>role_code</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>varchar(100)</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D8" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E8" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" s="18" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="17" t="inlineStr">
         <is>
           <t>화면ID:액션 형식  ·  화면ID=[A-Z]{4}M[0-9]{3}  ·  액션=inqy(조회)/sv(저장)/cnfr(확정)/aprl(승인)/prt(출력)</t>
         </is>
       </c>
-      <c r="G8" s="16" t="inlineStr">
+      <c r="G8" s="15" t="inlineStr">
         <is>
           <t>필요 권한 코드(화면ID:액션). 외부 권한API의 사용자 화면권한(Y/N)과 AND 비교</t>
         </is>
       </c>
-      <c r="H8" s="16" t="inlineStr">
+      <c r="H8" s="15" t="inlineStr">
         <is>
           <t>CLSGM001:inqy</t>
         </is>
@@ -6101,7 +6087,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>범례: 유효값(코드값) 열=코드성 컬럼만 기재(연녹 음영) · PK 컬럼 음영 · [핵심 로직]=실행/조회 분기에 사용 · '-'=자유값/해당없음</t>
         </is>
@@ -6149,162 +6135,162 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>테이블 ID</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>business_service.bs_client</t>
         </is>
       </c>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="13" t="inlineStr">
+      <c r="C2" s="13" t="n"/>
+      <c r="D2" s="13" t="n"/>
+      <c r="E2" s="13" t="n"/>
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>논리명</t>
         </is>
       </c>
-      <c r="G2" s="14" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>호출 Client 등록</t>
         </is>
       </c>
-      <c r="H2" s="14" t="n"/>
+      <c r="H2" s="13" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>주요 Key</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>client_id</t>
         </is>
       </c>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="12" t="inlineStr">
         <is>
           <t>DBMS</t>
         </is>
       </c>
-      <c r="G3" s="14" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>PostgreSQL</t>
         </is>
       </c>
-      <c r="H3" s="14" t="n"/>
+      <c r="H3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>서비스를 호출하는 Client(채널) 등록(§5.2 X-Client-ID)</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="14" t="n"/>
-      <c r="E4" s="14" t="n"/>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="13" t="n"/>
+      <c r="E4" s="13" t="n"/>
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>출처</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>상세설계서 v1.3 §7.2 (신규)</t>
         </is>
       </c>
-      <c r="H4" s="14" t="n"/>
+      <c r="H4" s="13" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>컬럼 ID</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>타입</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Not Null</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="F6" s="15" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>유효값(코드값)</t>
         </is>
       </c>
-      <c r="G6" s="15" t="inlineStr">
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>용도</t>
         </is>
       </c>
-      <c r="H6" s="15" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>예시</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>client_id</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>varchar(80)</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E7" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="18" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="17" t="inlineStr">
         <is>
           <t>형식 {채널}-{시스템}-{일련번호}  ·  정규식 [A-Z0-9]+-[A-Z0-9]+-[0-9]{2}  ·  채널은 하이픈 없는 코드</t>
         </is>
       </c>
-      <c r="G7" s="16" t="inlineStr">
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>호출 Client 식별자(X-Client-ID). 명명규칙 {채널}-{시스템}-{일련번호} [핵심 로직]</t>
         </is>
       </c>
-      <c r="H7" s="16" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
         <is>
           <t>MCP-IFRS17-01</t>
         </is>
@@ -6370,7 +6356,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F9" s="18" t="inlineStr">
+      <c r="F9" s="17" t="inlineStr">
         <is>
           <t>MCP, AI-AGENT, BATCH 등</t>
         </is>
@@ -6442,7 +6428,7 @@
           <t>'Y'</t>
         </is>
       </c>
-      <c r="F11" s="18" t="inlineStr">
+      <c r="F11" s="17" t="inlineStr">
         <is>
           <t>Y(사용), N(미사용)</t>
         </is>
@@ -6535,7 +6521,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>범례: 유효값(코드값) 열=코드성 컬럼만 기재(연녹 음영) · PK 컬럼 음영 · [핵심 로직]=실행/조회 분기에 사용 · '-'=자유값/해당없음</t>
         </is>
@@ -6583,204 +6569,204 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>테이블 ID</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>business_service.bs_client_service</t>
         </is>
       </c>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="13" t="inlineStr">
+      <c r="C2" s="13" t="n"/>
+      <c r="D2" s="13" t="n"/>
+      <c r="E2" s="13" t="n"/>
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>논리명</t>
         </is>
       </c>
-      <c r="G2" s="14" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>Client별 호출 허용</t>
         </is>
       </c>
-      <c r="H2" s="14" t="n"/>
+      <c r="H2" s="13" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>주요 Key</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>client_id + service_id</t>
         </is>
       </c>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="12" t="inlineStr">
         <is>
           <t>DBMS</t>
         </is>
       </c>
-      <c r="G3" s="14" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>PostgreSQL</t>
         </is>
       </c>
-      <c r="H3" s="14" t="n"/>
+      <c r="H3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Client가 호출 가능한 서비스 매핑(허용 목록)</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="14" t="n"/>
-      <c r="E4" s="14" t="n"/>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="13" t="n"/>
+      <c r="E4" s="13" t="n"/>
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>출처</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>상세설계서 v1.3 §7.2 (신규)</t>
         </is>
       </c>
-      <c r="H4" s="14" t="n"/>
+      <c r="H4" s="13" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>컬럼 ID</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>타입</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Not Null</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="F6" s="15" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>유효값(코드값)</t>
         </is>
       </c>
-      <c r="G6" s="15" t="inlineStr">
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>용도</t>
         </is>
       </c>
-      <c r="H6" s="15" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>예시</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>client_id</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>varchar(80)</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E7" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="16" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>Client ID(FK→BS_CLIENT)</t>
         </is>
       </c>
-      <c r="H7" s="16" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
         <is>
           <t>MCP-IFRS17-01</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>service_id</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>varchar(100)</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D8" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E8" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G8" s="16" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
         <is>
           <t>서비스 ID(FK→BS_SERVICE)</t>
         </is>
       </c>
-      <c r="H8" s="16" t="inlineStr">
+      <c r="H8" s="15" t="inlineStr">
         <is>
           <t>IFRS17.CLOSING.STATUS</t>
         </is>
@@ -6808,7 +6794,7 @@
           <t>'Y'</t>
         </is>
       </c>
-      <c r="F9" s="18" t="inlineStr">
+      <c r="F9" s="17" t="inlineStr">
         <is>
           <t>Y(허용), N(차단)</t>
         </is>
@@ -6901,7 +6887,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>범례: 유효값(코드값) 열=코드성 컬럼만 기재(연녹 음영) · PK 컬럼 음영 · [핵심 로직]=실행/조회 분기에 사용 · '-'=자유값/해당없음</t>
         </is>
@@ -6949,162 +6935,162 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>테이블 ID</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>business_service.bs_call_log</t>
         </is>
       </c>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="13" t="inlineStr">
+      <c r="C2" s="13" t="n"/>
+      <c r="D2" s="13" t="n"/>
+      <c r="E2" s="13" t="n"/>
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>논리명</t>
         </is>
       </c>
-      <c r="G2" s="14" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>호출 감사로그</t>
         </is>
       </c>
-      <c r="H2" s="14" t="n"/>
+      <c r="H2" s="13" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>주요 Key</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>request_id</t>
         </is>
       </c>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="12" t="inlineStr">
         <is>
           <t>DBMS</t>
         </is>
       </c>
-      <c r="G3" s="14" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>PostgreSQL</t>
         </is>
       </c>
-      <c r="H3" s="14" t="n"/>
+      <c r="H3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>서비스 호출 감사로그(§6.3). request_id(PK)는 서버 생성 유일값, 호출자 X-Request-ID는 client_request_id에 별도 저장(무결성)</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="14" t="n"/>
-      <c r="E4" s="14" t="n"/>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="13" t="n"/>
+      <c r="E4" s="13" t="n"/>
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>출처</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>상세설계서 v1.3 §7.3 (원본) + 감사 무결성 보강</t>
         </is>
       </c>
-      <c r="H4" s="14" t="n"/>
+      <c r="H4" s="13" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>컬럼 ID</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>타입</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Not Null</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="F6" s="15" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>유효값(코드값)</t>
         </is>
       </c>
-      <c r="G6" s="15" t="inlineStr">
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>용도</t>
         </is>
       </c>
-      <c r="H6" s="15" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>예시</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>request_id</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>varchar(80)</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E7" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="16" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>호출 요청 고유 ID — 서버 생성 유일값(호출자 헤더 미사용). 코드 반영 예정 [핵심 로직]</t>
         </is>
       </c>
-      <c r="H7" s="16" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
         <is>
           <t>REQ-20260714093012345-1</t>
         </is>
@@ -7488,7 +7474,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F18" s="18" t="inlineStr">
+      <c r="F18" s="17" t="inlineStr">
         <is>
           <t>COMPLETED, PARTIAL, FAILED 등 (부록D)</t>
         </is>
@@ -7522,7 +7508,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F19" s="18" t="inlineStr">
+      <c r="F19" s="17" t="inlineStr">
         <is>
           <t>200, 400, 401, 403, 404, 500 등</t>
         </is>
@@ -7556,7 +7542,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F20" s="18" t="inlineStr">
+      <c r="F20" s="17" t="inlineStr">
         <is>
           <t>BS-VAL-001, BS-AUTH-003 등 (부록A)</t>
         </is>
@@ -7743,7 +7729,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="12" t="inlineStr">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>범례: 유효값(코드값) 열=코드성 컬럼만 기재(연녹 음영) · PK 컬럼 음영 · [핵심 로직]=실행/조회 분기에 사용 · '-'=자유값/해당없음</t>
         </is>
@@ -7791,246 +7777,246 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>테이블 ID</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>business_service.bs_access_entity</t>
         </is>
       </c>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="13" t="inlineStr">
+      <c r="C2" s="13" t="n"/>
+      <c r="D2" s="13" t="n"/>
+      <c r="E2" s="13" t="n"/>
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>논리명</t>
         </is>
       </c>
-      <c r="G2" s="14" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>접근 업무객체 이력</t>
         </is>
       </c>
-      <c r="H2" s="14" t="n"/>
+      <c r="H2" s="13" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>주요 Key</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>request_id + entity_type + entity_id</t>
         </is>
       </c>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="12" t="inlineStr">
         <is>
           <t>DBMS</t>
         </is>
       </c>
-      <c r="G3" s="14" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>PostgreSQL</t>
         </is>
       </c>
-      <c r="H3" s="14" t="n"/>
+      <c r="H3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>호출별 접근 업무객체 이력(§6.3 accessed_entity_ids)</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="14" t="n"/>
-      <c r="E4" s="14" t="n"/>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="13" t="n"/>
+      <c r="E4" s="13" t="n"/>
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>출처</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>상세설계서 v1.3 §7.2 (신규)</t>
         </is>
       </c>
-      <c r="H4" s="14" t="n"/>
+      <c r="H4" s="13" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>컬럼 ID</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>타입</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Not Null</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="F6" s="15" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>유효값(코드값)</t>
         </is>
       </c>
-      <c r="G6" s="15" t="inlineStr">
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>용도</t>
         </is>
       </c>
-      <c r="H6" s="15" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>예시</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>request_id</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>varchar(80)</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E7" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="16" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>호출 요청 ID(FK→BS_CALL_LOG)</t>
         </is>
       </c>
-      <c r="H7" s="16" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
         <is>
           <t>REQ-20260714-0001</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>entity_type</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>varchar(50)</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D8" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E8" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G8" s="16" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
         <is>
           <t>접근 객체 유형</t>
         </is>
       </c>
-      <c r="H8" s="16" t="inlineStr">
+      <c r="H8" s="15" t="inlineStr">
         <is>
           <t>CLOSING</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>entity_id</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>varchar(200)</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D9" s="17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E9" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F9" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G9" s="16" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G9" s="15" t="inlineStr">
         <is>
           <t>접근 객체 식별자</t>
         </is>
       </c>
-      <c r="H9" s="16" t="inlineStr">
+      <c r="H9" s="15" t="inlineStr">
         <is>
           <t>2026-06</t>
         </is>
@@ -8075,7 +8061,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>범례: 유효값(코드값) 열=코드성 컬럼만 기재(연녹 음영) · PK 컬럼 음영 · [핵심 로직]=실행/조회 분기에 사용 · '-'=자유값/해당없음</t>
         </is>

</xml_diff>

<commit_message>
docs: BS_SERVICE 정합성 보완 (domain/owner nullable, CON-01에 service_type 추가)
테이블-화면 정합성 대조 결과 반영:
- schema.sql/별첨C: domain_code·owner_department NOT NULL 제거(nullable)
  (로직 미사용·표시용 컬럼)
- 별첨D CON-01: 서비스 유형(service_type) 필드 추가 - 필드명세 행 +
  샘플 목업 라디오(READ/ACTION) 이미지 재캡쳐
- 개정이력: 별첨C v1.4, 별첨D v1.2 추가

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SLMxyQgKYFz74Rk29M4m6g
</commit_message>
<xml_diff>
--- a/docs/별첨C_테이블설계서.xlsx
+++ b/docs/별첨C_테이블설계서.xlsx
@@ -552,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -708,6 +708,33 @@
       <c r="E8" s="5" t="inlineStr">
         <is>
           <t>사용 6 / 미사용 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>v1.4</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>DBInc</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>BS_SERVICE domain_code·owner_department NOT NULL 제거(nullable)</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>로직 미사용·표시용 컬럼 완화</t>
         </is>
       </c>
     </row>
@@ -5037,11 +5064,7 @@
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr"/>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D10" s="4" t="inlineStr"/>
       <c r="E10" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -5054,7 +5077,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>업무 도메인 분류 코드(표시용)</t>
+          <t>업무 도메인 분류 코드(표시용, 로직 미사용). nullable</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -5092,7 +5115,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>서비스 성격. 등록 시 값 검증에만 사용</t>
+          <t>서비스 성격. 등록 시 값 검증(CON-01 필수 입력)</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -5151,11 +5174,7 @@
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr"/>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D13" s="4" t="inlineStr"/>
       <c r="E13" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -5168,7 +5187,7 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>서비스 업무 책임 부서(Owner)</t>
+          <t>서비스 업무 책임 부서(Owner, 표시용). nullable</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">

</xml_diff>